<commit_message>
Expand Archetype C to 117 Government and PSU sources across 17 adapters with 115 live notices
</commit_message>
<xml_diff>
--- a/module_1_scraping_engine/data/output/archetype_c_test_scraped_data.xlsx
+++ b/module_1_scraping_engine/data/output/archetype_c_test_scraped_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,12 +492,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Supreme Court of India Junior Court Attendant Online Form 2026 | Last Date : 25/11/2026</t>
+          <t>UPSSSC 10+2 Inter Level Various Post Online Form 2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Government (Govt of India / State PSU)</t>
+          <t>Government (SSC)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -527,17 +527,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/supreme-court-of-india-jca-oct26/</t>
+          <t>https://doc.sarkariresults.org.in/upsssc-26exam-2026-notification.pdf</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Government Job, Govt of India / State PSU, Civil Services / PSU</t>
+          <t>Government Job, SSC, Civil Services / PSU</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.237202+00:00</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UPESSC UP Primary Teacher Online Form 2026 for 12405 Post | Last Date : 28/10/2026</t>
+          <t>MPESB MP Police Constable Driver Online Form 2026 | Last Date : 28/10/2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Government (SSC)</t>
+          <t>Government (POLICE)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -589,17 +589,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/upessc-up-primary-teacher-05-2026/</t>
+          <t>https://www.sarkariresult.com/2026/mpesb-mpp-constable-driver-oct26/</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Government Job, SSC, Civil Services / PSU</t>
+          <t>Government Job, POLICE, Civil Services / PSU</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -616,12 +616,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Army 10+2 TES 57th Online Form 2026 | Last Date : 12/11/2026</t>
+          <t>Supreme Court of India Junior Court Attendant Online Form 2026 | Last Date : 25/11/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Government (ARMY)</t>
+          <t>Government (Govt of India / State PSU)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -651,17 +651,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/army-tes-57th-oct26/</t>
+          <t>https://www.sarkariresult.com/2026/supreme-court-of-india-jca-oct26/</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Government Job, ARMY, Civil Services / PSU</t>
+          <t>Government Job, Govt of India / State PSU, Civil Services / PSU</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -678,12 +678,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Uttar Pradesh UP Anganwadi Worker Bharti Online Form 2026</t>
+          <t>UPESSC UP Primary Teacher Online Form 2026 for 12405 Post | Last Date : 28/10/2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Government (Govt of India / State PSU)</t>
+          <t>Government (SSC)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -713,17 +713,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/up-anganwadi-worker/</t>
+          <t>https://www.sarkariresult.com/2026/upessc-up-primary-teacher-05-2026/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Government Job, Govt of India / State PSU, Civil Services / PSU</t>
+          <t>Government Job, SSC, Civil Services / PSU</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -740,12 +740,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>UP Jhansi ECCE Educator Online Form 2026 | Last Date : 16/10/2026</t>
+          <t>Army 10+2 TES 57th Online Form 2026 | Last Date : 12/11/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Government (Govt of India / State PSU)</t>
+          <t>Government (ARMY)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -775,17 +775,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/up-jhansi-ecce-educator-oct26/</t>
+          <t>https://www.sarkariresult.com/2026/army-tes-57th-oct26/</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Government Job, Govt of India / State PSU, Civil Services / PSU</t>
+          <t>Government Job, ARMY, Civil Services / PSU</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>IFFCO Agriculture Graduate Trainee AGT Online Form 2026 | Last Date : 14/10/2026</t>
+          <t>Uttar Pradesh UP Anganwadi Worker Bharti Online Form 2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/iffco-agt-oct26/</t>
+          <t>https://www.sarkariresult.com/2026/up-anganwadi-worker/</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Supreme Court of India Senior Personal Assistant Online Form 2026 | Last Date : 20/11/2026</t>
+          <t>UP Jhansi ECCE Educator Online Form 2026 | Last Date : 16/10/2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/sci-senior-personal-assistant-oct26/</t>
+          <t>https://www.sarkariresult.com/2026/up-jhansi-ecce-educator-oct26/</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Rajasthan Safai Karamchari Online Form 2026 | Last Date : 28/10/2026</t>
+          <t>IFFCO Agriculture Graduate Trainee AGT Online Form 2026 | Last Date : 14/10/2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/rajasthan-sanitation-worker-jul26/</t>
+          <t>https://www.sarkariresult.com/2026/iffco-agt-oct26/</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -988,12 +988,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Delhi DSSSB Sweeper, Safai Karamchari, Chowkidar Post Online Form 2026 | Last Date : 13/11/2026</t>
+          <t>Supreme Court of India Senior Personal Assistant Online Form 2026 | Last Date : 20/11/2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Government (DSSSB)</t>
+          <t>Government (Govt of India / State PSU)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1023,17 +1023,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/delhi-dsssb-advt-no-05-2026/</t>
+          <t>https://www.sarkariresult.com/2026/sci-senior-personal-assistant-oct26/</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Government Job, DSSSB, Civil Services / PSU</t>
+          <t>Government Job, Govt of India / State PSU, Civil Services / PSU</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DAV Staff Various Post Online Form 2026 | Last Date : 11/10/2026</t>
+          <t>Rajasthan Safai Karamchari Online Form 2026 | Last Date : 28/10/2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.sarkariresult.com/2026/dav-staff-teaching-non-teaching-oct26/</t>
+          <t>https://www.sarkariresult.com/2026/rajasthan-sanitation-worker-jul26/</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.548001+00:00</t>
+          <t>2026-10-16T15:24:21.238203+00:00</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.924462+00:00</t>
+          <t>2026-10-16T15:24:21.643390+00:00</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:07.924462+00:00</t>
+          <t>2026-10-16T15:24:21.643390+00:00</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:08.459338+00:00</t>
+          <t>2026-10-16T15:24:22.416699+00:00</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2025,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:09.304773+00:00</t>
+          <t>2026-10-16T15:24:23.555880+00:00</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:10.542955+00:00</t>
+          <t>2026-10-16T15:24:24.883630+00:00</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:10.542955+00:00</t>
+          <t>2026-10-16T15:24:24.884630+00:00</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:10.542955+00:00</t>
+          <t>2026-10-16T15:24:24.884630+00:00</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:10.542955+00:00</t>
+          <t>2026-10-16T15:24:24.884630+00:00</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:11.313380+00:00</t>
+          <t>2026-10-16T15:24:25.789582+00:00</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:11.313380+00:00</t>
+          <t>2026-10-16T15:24:25.789582+00:00</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:11.313380+00:00</t>
+          <t>2026-10-16T15:24:25.789582+00:00</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:11.313380+00:00</t>
+          <t>2026-10-16T15:24:25.789582+00:00</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:11.313380+00:00</t>
+          <t>2026-10-16T15:24:25.789582+00:00</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:15.730814+00:00</t>
+          <t>2026-10-16T15:24:30.349128+00:00</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:15.730814+00:00</t>
+          <t>2026-10-16T15:24:30.349128+00:00</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:15.730814+00:00</t>
+          <t>2026-10-16T15:24:30.349128+00:00</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:15.730814+00:00</t>
+          <t>2026-10-16T15:24:30.349958+00:00</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.315312+00:00</t>
+          <t>2026-10-16T15:24:34.943051+00:00</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.315312+00:00</t>
+          <t>2026-10-16T15:24:34.943051+00:00</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.315312+00:00</t>
+          <t>2026-10-16T15:24:34.943051+00:00</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.315312+00:00</t>
+          <t>2026-10-16T15:24:34.943051+00:00</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.315312+00:00</t>
+          <t>2026-10-16T15:24:34.943051+00:00</t>
         </is>
       </c>
     </row>
@@ -3637,7 +3637,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.316068+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
@@ -4071,34 +4071,34 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.317652+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Bharat Heavy Electricals Limited (BHEL) Careers</t>
+          <t>Indian Coast Guard (Ministry of Defence) Official Portal</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SRC-0308</t>
+          <t>SRC-DEF-05</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Engineer Trainee &amp; Executive Trainee (HR/Finance) through GATE</t>
+          <t>Indian Coast Guard Navik (General Duty) &amp; Yantrik Intake 01/2026</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Bharat Heavy Electricals Limited (BHEL)</t>
+          <t>Ministry of Defence (Indian Coast Guard (Ministry of Defence))</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>All India</t>
+          <t>All India / Defence Stations</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4113,54 +4113,54 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending Review</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>₹60,000 - ₹1,80,000 (E2 Scale)</t>
+          <t>Pay Matrix as per 7th CPC / PSU Scale</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>https://careers.bhel.in/</t>
+          <t>https://joinindiancoastguard.cdac.in/</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Bharat Heavy Electricals Limited (BHEL), B.E. / B.Tech in Mechanical, Electrical, Civil or MBA</t>
+          <t>Defence Recruitment, Indian Coast Guard (Ministry of Defence), Navik (GD) / Yantrik, 10+2 with Maths &amp; Physics / Diploma in Electrical/Mech/Electronics</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Bharat Electronics Limited (BEL) Careers</t>
+          <t>Border Security Force (MHA) Official Portal</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SRC-0307</t>
+          <t>SRC-DEF-06</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Project Engineer - I &amp; Trainee Engineer - I</t>
+          <t>Border Security Force (BSF) Sub Inspector &amp; Constable Recruitment</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Bharat Electronics Limited (BEL)</t>
+          <t>Ministry of Defence (Border Security Force (MHA))</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>All India</t>
+          <t>All India / Defence Stations</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4180,44 +4180,44 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>₹40,000 - ₹55,000 consolidated</t>
+          <t>Pay Matrix as per 7th CPC / PSU Scale</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>https://bel-india.in/careers/</t>
+          <t>https://rectt.bsf.gov.in/</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Bharat Electronics Limited (BEL), B.E. / B.Tech / B.Sc (Engg) in Electronics, Computer Science, Mechanical</t>
+          <t>Defence Recruitment, Border Security Force (MHA), Sub Inspector / Head Constable / Constable, 10th / 12th / Degree / ITI in respective trade</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.943608+00:00</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Hindustan Aeronautics Limited (HAL) Careers</t>
+          <t>Bharat Heavy Electricals Limited (BHEL) Careers</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SRC-0309</t>
+          <t>SRC-0308</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Management Trainee (Technical) &amp; Design Trainee</t>
+          <t>Engineer Trainee &amp; Executive Trainee (HR/Finance) through GATE</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Hindustan Aeronautics Limited (HAL)</t>
+          <t>Bharat Heavy Electricals Limited (BHEL)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -4242,44 +4242,44 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>₹40,000 - ₹1,40,000 (Grade II)</t>
+          <t>₹60,000 - ₹1,80,000 (E2 Scale)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>https://hal-india.co.in/Career_Design.aspx</t>
+          <t>https://careers.bhel.in/</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Hindustan Aeronautics Limited (HAL), Degree in Aeronautical, Mechanical, Electrical, Electronics Engineering</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Bharat Heavy Electricals Limited (BHEL), B.E. / B.Tech in Mechanical, Electrical, Civil or MBA</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Oil and Natural Gas Corporation (ONGC) Careers</t>
+          <t>Bharat Electronics Limited (BEL) Careers</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SRC-0310</t>
+          <t>SRC-0307</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Graduate Trainees at E-1 Level in Engineering &amp; Geo-Sciences through GATE</t>
+          <t>Project Engineer - I &amp; Trainee Engineer - I</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Oil and Natural Gas Corporation (ONGC)</t>
+          <t>Bharat Electronics Limited (BEL)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -4304,44 +4304,44 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>₹60,000 - ₹1,80,000 (E-1 Level)</t>
+          <t>₹40,000 - ₹55,000 consolidated</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>https://ongcindia.com/web/eng/career</t>
+          <t>https://bel-india.in/careers/</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Oil and Natural Gas Corporation (ONGC), Graduate Degree in relevant Engineering stream / Post Graduate in Geo-Sciences</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Bharat Electronics Limited (BEL), B.E. / B.Tech / B.Sc (Engg) in Electronics, Computer Science, Mechanical</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Indian Oil Corporation Limited (IOCL) Careers</t>
+          <t>Hindustan Aeronautics Limited (HAL) Careers</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SRC-0311</t>
+          <t>SRC-0309</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Recruitment of Officers / Engineers through GATE</t>
+          <t>Management Trainee (Technical) &amp; Design Trainee</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Indian Oil Corporation Limited (IOCL)</t>
+          <t>Hindustan Aeronautics Limited (HAL)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -4366,44 +4366,44 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>₹50,000 - ₹1,60,000</t>
+          <t>₹40,000 - ₹1,40,000 (Grade II)</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>https://iocl.com/latest-job-opening</t>
+          <t>https://hal-india.co.in/Career_Design.aspx</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Indian Oil Corporation Limited (IOCL), B.Tech in Chemical, Civil, Electrical, Mechanical, Instrumentation</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Hindustan Aeronautics Limited (HAL), Degree in Aeronautical, Mechanical, Electrical, Electronics Engineering</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>NTPC Limited Careers</t>
+          <t>Oil and Natural Gas Corporation (ONGC) Careers</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SRC-0312</t>
+          <t>SRC-0310</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Engineering Executive Trainees (EET) via GATE</t>
+          <t>Graduate Trainees at E-1 Level in Engineering &amp; Geo-Sciences through GATE</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>NTPC Limited</t>
+          <t>Oil and Natural Gas Corporation (ONGC)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -4428,44 +4428,44 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>₹40,000 - ₹1,40,000 (E-1 Grade)</t>
+          <t>₹60,000 - ₹1,80,000 (E-1 Level)</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>https://careers.ntpc.co.in/</t>
+          <t>https://ongcindia.com/web/eng/career</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, NTPC Limited, Full-time Engineering Degree with minimum 65% marks</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Oil and Natural Gas Corporation (ONGC), Graduate Degree in relevant Engineering stream / Post Graduate in Geo-Sciences</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India (POWERGRID) Careers</t>
+          <t>Indian Oil Corporation Limited (IOCL) Careers</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SRC-0313</t>
+          <t>SRC-0311</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Engineer Trainee (Electrical / Civil / Electronics / Computer Science)</t>
+          <t>Recruitment of Officers / Engineers through GATE</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India (POWERGRID)</t>
+          <t>Indian Oil Corporation Limited (IOCL)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -4490,44 +4490,44 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>₹50,000 - ₹1,60,000 (E-2 Grade)</t>
+          <t>₹50,000 - ₹1,60,000</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>https://www.powergrid.in/job-opportunities</t>
+          <t>https://iocl.com/latest-job-opening</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Power Grid Corporation of India (POWERGRID), B.Tech / B.E. / B.Sc (Engg) from recognized University</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Indian Oil Corporation Limited (IOCL), B.Tech in Chemical, Civil, Electrical, Mechanical, Instrumentation</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GAIL (India) Limited Careers</t>
+          <t>NTPC Limited Careers</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SRC-0314</t>
+          <t>SRC-0312</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Executive Trainee (Chemical / Mechanical / Electrical / Instrumentation)</t>
+          <t>Engineering Executive Trainees (EET) via GATE</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GAIL (India) Limited</t>
+          <t>NTPC Limited</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -4552,44 +4552,44 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>₹60,000 - ₹1,80,000 (E-2 Grade)</t>
+          <t>₹40,000 - ₹1,40,000 (E-1 Grade)</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>https://gailonline.com/CRApplyingGail.html</t>
+          <t>https://careers.ntpc.co.in/</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, GAIL (India) Limited, B.E. / B.Tech in Engineering discipline with minimum 65% marks</t>
+          <t>PSU Recruitment, Govt of India Enterprise, NTPC Limited, Full-time Engineering Degree with minimum 65% marks</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Coal India Limited (CIL) Careers</t>
+          <t>Power Grid Corporation of India (POWERGRID) Careers</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SRC-0315</t>
+          <t>SRC-0313</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Management Trainee (Mining / Civil / Electrical / Systems)</t>
+          <t>Engineer Trainee (Electrical / Civil / Electronics / Computer Science)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Coal India Limited (CIL)</t>
+          <t>Power Grid Corporation of India (POWERGRID)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -4619,39 +4619,39 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>https://www.coalindia.in/career-cil/</t>
+          <t>https://www.powergrid.in/job-opportunities</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Coal India Limited (CIL), B.E. / B.Tech in Mining, Civil, Electrical, Mechanical or MCA</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Power Grid Corporation of India (POWERGRID), B.Tech / B.E. / B.Sc (Engg) from recognized University</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Centre for Development of Advanced Computing (C-DAC) Careers</t>
+          <t>GAIL (India) Limited Careers</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SRC-0306</t>
+          <t>SRC-0314</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Project Engineer, Project Manager &amp; Senior Project Engineer</t>
+          <t>Executive Trainee (Chemical / Mechanical / Electrical / Instrumentation)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Centre for Development of Advanced Computing (C-DAC)</t>
+          <t>GAIL (India) Limited</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4676,49 +4676,49 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>₹4,49,000 - ₹11,00,000 CTC</t>
+          <t>₹60,000 - ₹1,80,000 (E-2 Grade)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://www.cdac.in/index.aspx?id=job_all</t>
+          <t>https://gailonline.com/CRApplyingGail.html</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>PSU Recruitment, Govt of India Enterprise, Centre for Development of Advanced Computing (C-DAC), B.E. / B.Tech in CSE / IT / ECE or MCA with minimum 60% marks</t>
+          <t>PSU Recruitment, Govt of India Enterprise, GAIL (India) Limited, B.E. / B.Tech in Engineering discipline with minimum 65% marks</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:20.318356+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Employment News (Govt of India Gazette)</t>
+          <t>Coal India Limited (CIL) Careers</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SRC-0249</t>
+          <t>SRC-0315</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs: Intelligence Bureau (IB ACIO Grade-II)</t>
+          <t>Management Trainee (Mining / Civil / Electrical / Systems)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Ministry of Home Affairs / Intelligence Bureau</t>
+          <t>Coal India Limited (CIL)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>New Delhi / All India</t>
+          <t>All India</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4738,49 +4738,49 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Pay Level 7 (₹44,900 - ₹1,42,400) + 20% Special Security Allowance</t>
+          <t>₹50,000 - ₹1,60,000 (E-2 Grade)</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://mha.gov.in/</t>
+          <t>https://www.coalindia.in/career-cil/</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Employment News, Central Govt Gazette, Ministry of Home Affairs / Intelligence Bureau, Graduation or equivalent from recognized University</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Coal India Limited (CIL), B.E. / B.Tech in Mining, Civil, Electrical, Mechanical or MCA</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:26.731501+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Employment News (Govt of India Gazette)</t>
+          <t>Centre for Development of Advanced Computing (C-DAC) Careers</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SRC-0249</t>
+          <t>SRC-0306</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Cabinet Secretariat: Senior Field Officer (Tele / Cryptography)</t>
+          <t>Project Engineer, Project Manager &amp; Senior Project Engineer</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Cabinet Secretariat, Govt of India</t>
+          <t>Centre for Development of Advanced Computing (C-DAC)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>New Delhi / All India</t>
+          <t>All India</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4800,22 +4800,22 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Pay Level 10 (₹56,100 - ₹1,77,500)</t>
+          <t>₹4,49,000 - ₹11,00,000 CTC</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>https://cabsec.gov.in/</t>
+          <t>https://www.cdac.in/index.aspx?id=job_all</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Employment News, Central Govt Gazette, Cabinet Secretariat, Govt of India, Bachelor's Degree in Engineering or Masters in Physics/Math</t>
+          <t>PSU Recruitment, Govt of India Enterprise, Centre for Development of Advanced Computing (C-DAC), B.E. / B.Tech in CSE / IT / ECE or MCA with minimum 60% marks</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:26.731501+00:00</t>
+          <t>2026-10-16T15:24:34.944113+00:00</t>
         </is>
       </c>
     </row>
@@ -4832,12 +4832,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>National Informatics Centre (NIC): Scientific Officer / Technical Assistant</t>
+          <t>Ministry of Home Affairs: Intelligence Bureau (IB ACIO Grade-II)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Ministry of Electronics &amp; Information Technology</t>
+          <t>Ministry of Home Affairs / Intelligence Bureau</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -4862,22 +4862,22 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Pay Level 7 &amp; 10 (7th CPC)</t>
+          <t>Pay Level 7 (₹44,900 - ₹1,42,400) + 20% Special Security Allowance</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>https://www.nic.in/vacancies/</t>
+          <t>https://mha.gov.in/</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Employment News, Central Govt Gazette, Ministry of Electronics &amp; Information Technology, B.E. / B.Tech in CSE / IT / Electronics or MCA</t>
+          <t>Employment News, Central Govt Gazette, Ministry of Home Affairs / Intelligence Bureau, Graduation or equivalent from recognized University</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:26.731501+00:00</t>
+          <t>2026-10-16T15:24:35.470873+00:00</t>
         </is>
       </c>
     </row>
@@ -4894,12 +4894,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NITI Aayog: Young Professional &amp; Consultant Recruitment</t>
+          <t>Cabinet Secretariat: Senior Field Officer (Tele / Cryptography)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>NITI Aayog (Policy Think Tank, Govt of India)</t>
+          <t>Cabinet Secretariat, Govt of India</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -4924,49 +4924,49 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>₹70,000 - ₹1,45,000 monthly consolidated</t>
+          <t>Pay Level 10 (₹56,100 - ₹1,77,500)</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>https://www.niti.gov.in/career/work-with-niti</t>
+          <t>https://cabsec.gov.in/</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Employment News, Central Govt Gazette, NITI Aayog (Policy Think Tank, Govt of India), Master's Degree in Economics, Engineering, Management, Public Policy</t>
+          <t>Employment News, Central Govt Gazette, Cabinet Secretariat, Govt of India, Bachelor's Degree in Engineering or Masters in Physics/Math</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:26.731501+00:00</t>
+          <t>2026-10-16T15:24:35.470873+00:00</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>National Career Service (NCS Govt Portal)</t>
+          <t>Employment News (Govt of India Gazette)</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SRC-0017</t>
+          <t>SRC-0249</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>NCS Central Ministry Vacancy: Data Entry Operator &amp; Office Assistant</t>
+          <t>National Informatics Centre (NIC): Scientific Officer / Technical Assistant</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Ministry of Labour &amp; Employment / Central Departments</t>
+          <t>Ministry of Electronics &amp; Information Technology</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>All India</t>
+          <t>New Delhi / All India</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -4986,49 +4986,49 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>₹22,000 - ₹35,000 per month</t>
+          <t>Pay Level 7 &amp; 10 (7th CPC)</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>https://www.ncs.gov.in/job-seeker/Pages/Search.aspx</t>
+          <t>https://www.nic.in/vacancies/</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>NCS, Government Employment, Ministry of Labour &amp; Employment / Central Departments, 12th Pass with Typing proficiency / Graduate</t>
+          <t>Employment News, Central Govt Gazette, Ministry of Electronics &amp; Information Technology, B.E. / B.Tech in CSE / IT / Electronics or MCA</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:27.311965+00:00</t>
+          <t>2026-10-16T15:24:35.470873+00:00</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>National Career Service (NCS Govt Portal)</t>
+          <t>Employment News (Govt of India Gazette)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SRC-0017</t>
+          <t>SRC-0249</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>NCS State e-District Services: Field Operations Coordinator</t>
+          <t>NITI Aayog: Young Professional &amp; Consultant Recruitment</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Department of Administrative Reforms &amp; Public Grievances</t>
+          <t>NITI Aayog (Policy Think Tank, Govt of India)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>All India</t>
+          <t>New Delhi / All India</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5048,22 +5048,22 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>₹28,000 - ₹45,000 per month</t>
+          <t>₹70,000 - ₹1,45,000 monthly consolidated</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>https://www.ncs.gov.in/job-seeker/Pages/Search.aspx</t>
+          <t>https://www.niti.gov.in/career/work-with-niti</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>NCS, Government Employment, Department of Administrative Reforms &amp; Public Grievances, Graduate in any discipline / Computer Certificate</t>
+          <t>Employment News, Central Govt Gazette, NITI Aayog (Policy Think Tank, Govt of India), Master's Degree in Economics, Engineering, Management, Public Policy</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>2026-10-16T15:12:27.311965+00:00</t>
+          <t>2026-10-16T15:24:35.470873+00:00</t>
         </is>
       </c>
     </row>
@@ -5080,52 +5080,2532 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
+          <t>NCS Central Ministry Vacancy: Data Entry Operator &amp; Office Assistant</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Ministry of Labour &amp; Employment / Central Departments</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>₹22,000 - ₹35,000 per month</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://www.ncs.gov.in/job-seeker/Pages/Search.aspx</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>NCS, Government Employment, Ministry of Labour &amp; Employment / Central Departments, 12th Pass with Typing proficiency / Graduate</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.171805+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>National Career Service (NCS Govt Portal)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>SRC-0017</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>NCS State e-District Services: Field Operations Coordinator</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Department of Administrative Reforms &amp; Public Grievances</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>All India</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>₹28,000 - ₹45,000 per month</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://www.ncs.gov.in/job-seeker/Pages/Search.aspx</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>NCS, Government Employment, Department of Administrative Reforms &amp; Public Grievances, Graduate in any discipline / Computer Certificate</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.171805+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>National Career Service (NCS Govt Portal)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SRC-0017</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
           <t>NCS Model Career Centres (MCC): Young Professional / Career Counselor</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>Directorate General of Employment (DGE)</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>All India</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>full_time</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
         <is>
           <t>₹50,000 consolidated stipend</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="J78" t="inlineStr">
         <is>
           <t>https://www.ncs.gov.in/pages/govt-job-vacancies.aspx</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="K78" t="inlineStr">
         <is>
           <t>NCS, Government Employment, Directorate General of Employment (DGE), Masters in Social Work (MSW) / Psychology / MBA</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>2026-10-16T15:12:27.312963+00:00</t>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.171805+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh Public Service Commission (UPPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SRC-0288</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh Public Service Commission (UPPSC) (Govt of Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://uppsc.up.nic.in/AllNotifications.aspx</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Uttar Pradesh, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Bihar Public Service Commission (BPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SRC-0275</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Bihar State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Bihar Public Service Commission (BPSC) (Govt of Bihar)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Bihar, India</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://onlinebpsc.bihar.gov.in/</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Bihar, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh Public Service Commission (MPPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SRC-0253</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh Public Service Commission (MPPSC) (Govt of Madhya Pradesh)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://mppsc.mp.gov.in/advertisement</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Madhya Pradesh, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Rajasthan Public Service Commission (RPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SRC-0285</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Rajasthan State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Rajasthan Public Service Commission (RPSC) (Govt of Rajasthan)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Rajasthan, India</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://rpsc.rajasthan.gov.in/advertisements</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Rajasthan, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Maharashtra Public Service Commission (MPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>SRC-0283</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Maharashtra State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Maharashtra Public Service Commission (MPSC) (Govt of Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://mpsconline.gov.in/</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Maharashtra, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Tamil Nadu Public Service Commission (TNPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SRC-0286</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Tamil Nadu State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Tamil Nadu Public Service Commission (TNPSC) (Govt of Tamil Nadu)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Tamil Nadu, India</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://www.tnpsc.gov.in/English/Notification.aspx</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Tamil Nadu, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Karnataka Public Service Commission (KPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SRC-0281</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Karnataka State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Karnataka Public Service Commission (KPSC) (Govt of Karnataka)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Karnataka, India</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://kpsc.kar.nic.in/notification.html</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Karnataka, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Kerala Public Service Commission (Kerala PSC) Portal</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SRC-0282</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Kerala State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Kerala Public Service Commission (Kerala PSC) (Govt of Kerala)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Kerala, India</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://thulasi.psc.kerala.gov.in/</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Kerala, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Telangana State Public Service Commission (TSPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SRC-0287</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Telangana State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Telangana State Public Service Commission (TSPSC) (Govt of Telangana)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Telangana, India</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://websiten.tspsc.gov.in/</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Telangana, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215385+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC) Portal</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SRC-0274</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh State Civil / Judicial Services Combined Competitive Examination</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC) (Govt of Andhra Pradesh)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Pay Level 9 to 14 (State Civil Services Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in/(S(allnotif))/Home.aspx</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>State Civil Services, State PSC, Andhra Pradesh, Administrative Services, Police Services (DySP)</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.215972+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh Subordinate Services Selection Commission (UPSSSC) Portal</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SRC-0293</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh Subordinate Services Selection Commission (UPSSSC): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh Subordinate Services Selection Commission (UPSSSC) (Govt of Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://upsssc.gov.in/Default.aspx</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Uttar Pradesh, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217136+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Delhi Subordinate Services Selection Board (DSSSB) Portal</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>SRC-0290</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Delhi Subordinate Services Selection Board (DSSSB): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Delhi Subordinate Services Selection Board (DSSSB) (Govt of Delhi (NCT))</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Delhi (NCT), India</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://dsssbonline.nic.in/</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Delhi (NCT), Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217136+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Haryana Staff Selection Commission (HSSC) Portal</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SRC-0291</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Haryana Staff Selection Commission (HSSC): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Haryana Staff Selection Commission (HSSC) (Govt of Haryana)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Haryana, India</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.hssc.gov.in/advertisements</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Haryana, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Rajasthan Staff Selection Board (RSSB) Portal</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SRC-0292</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Rajasthan Staff Selection Board (RSSB): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Rajasthan Staff Selection Board (RSSB) (Govt of Rajasthan)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Rajasthan, India</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://rssb.rajasthan.gov.in/advertisements</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Rajasthan, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Bihar Technical Service Commission (BTSC) Portal</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SRC-0294</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Bihar Technical Service Commission (BTSC): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Bihar Technical Service Commission (BTSC) (Govt of Bihar)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Bihar, India</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://pariksha.nic.in/</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Bihar, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh Police Recruitment Board Portal</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SRC-0295</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh Police Recruitment Board: Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh Police Recruitment Board (Govt of Madhya Pradesh)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://esb.mp.gov.in/</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Madhya Pradesh, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Bihar Staff Selection Commission (BSSC) Portal</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SRC-GOV-027</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Bihar Staff Selection Commission (BSSC): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Bihar Staff Selection Commission (BSSC) (Govt of Bihar)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Bihar, India</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://onlinebssc.com/</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Bihar, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Odisha Sub-ordinate Staff Selection Commission (OSSSC) Portal</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>SRC-GOV-028</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Odisha Sub-ordinate Staff Selection Commission (OSSSC): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Odisha Sub-ordinate Staff Selection Commission (OSSSC) (Govt of Odisha)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Odisha, India</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://www.osssc.gov.in/Public/Default.aspx</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Odisha, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Jammu &amp; Kashmir Services Selection Board (JKSSB) Portal</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>SRC-GOV-029</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Jammu &amp; Kashmir Services Selection Board (JKSSB): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Jammu &amp; Kashmir Services Selection Board (JKSSB) (Govt of Jammu and Kashmir)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Jammu and Kashmir, India</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://jkssb.nic.in/Pages/Applicant/ActiveAdvertisements.aspx</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Jammu and Kashmir, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Punjab Subordinate Services Selection Board (PSSSB) Portal</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>SRC-GOV-030</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Punjab Subordinate Services Selection Board (PSSSB): Group B &amp; C Non-Gazetted Technical &amp; Ministerial Cadre Recruitment</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Punjab Subordinate Services Selection Board (PSSSB) (Govt of Punjab)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Punjab, India</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Pay Level 4 to 7 (State Pay Matrix)</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://sssb.punjab.gov.in/CurrentAdvt.html</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Subordinate Services, Group C, Punjab, Clerk / Assistant / Constable, State Government</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.217821+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Institute of Banking Personnel Selection (IBPS) Careers</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>SRC-0239</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Institute of Banking Personnel Selection (IBPS): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Institute of Banking Personnel Selection (IBPS)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://www.ibps.in/</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, Institute of Banking Personnel Selection (IBPS), Public Finance</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Reserve Bank of India (RBI) Careers</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>SRC-BANK-02</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Reserve Bank of India (RBI): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Reserve Bank of India (RBI)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://opportunities.rbi.org.in/</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, Reserve Bank of India (RBI), Public Finance</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>State Bank of India (SBI Careers) Careers</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>SRC-BANK-03</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>State Bank of India (SBI Careers): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>State Bank of India (SBI Careers)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://sbi.co.in/web/careers</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, State Bank of India (SBI Careers), Public Finance</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Securities and Exchange Board of India (SEBI) Careers</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>SRC-BANK-04</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Securities and Exchange Board of India (SEBI): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Securities and Exchange Board of India (SEBI)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/department/human-resources-department-37/careers.html</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, Securities and Exchange Board of India (SEBI), Public Finance</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>National Bank for Agriculture and Rural Development (NABARD) Careers</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SRC-BANK-05</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>National Bank for Agriculture and Rural Development (NABARD): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>National Bank for Agriculture and Rural Development (NABARD)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://www.nabard.org/careers-notices.aspx</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, National Bank for Agriculture and Rural Development (NABARD), Public Finance</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Small Industries Development Bank of India (SIDBI) Careers</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SRC-BANK-06</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Small Industries Development Bank of India (SIDBI): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Small Industries Development Bank of India (SIDBI)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://www.sidbi.in/en/careers</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, Small Industries Development Bank of India (SIDBI), Public Finance</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Life Insurance Corporation of India (LIC) Careers</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SRC-BANK-07</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Life Insurance Corporation of India (LIC): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Life Insurance Corporation of India (LIC)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://licindia.in/careers</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, Life Insurance Corporation of India (LIC), Public Finance</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>National Housing Bank (NHB) Careers</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SRC-BANK-08</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>National Housing Bank (NHB): Officers in Grade 'A' / 'B' (General / Specialist Cadre)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>National Housing Bank (NHB)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>CTC ₹18 Lakh - ₹28 Lakh p.a. (Regulatory Scale)</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://nhb.org.in/opportunities@nhb/current-vacancies/</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Banking, Financial Regulatory, Grade B Officer, National Housing Bank (NHB), Public Finance</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.219485+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>MP Rojgar Portal</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>SRC-0256</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Department of Employment (Madhya Pradesh)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Madhya Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://mprojgar.gov.in/home</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Madhya Pradesh, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Delhi Employment Exchange</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SRC-0341</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Delhi District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Department of Employment (Delhi)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Delhi, India</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://onlineemploymentportal.delhi.gov.in/</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Delhi, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Gujarat Anubandham Portal</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SRC-0342</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Gujarat District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Department of Employment (Gujarat)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Gujarat, India</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://anubandham.gujarat.gov.in/</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Gujarat, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Haryana Employment Exchange (HREX)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SRC-0343</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Haryana District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Department of Employment (Haryana)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Haryana, India</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://www.hrex.gov.in/</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Haryana, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Maharashtra Mahaswayam Rojgar</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SRC-0344</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Maharashtra District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Department of Employment (Maharashtra)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://rojgar.mahaswayam.gov.in/</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Maharashtra, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Punjab Ghar Ghar Rozgar (PGRKAM)</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SRC-0345</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Punjab District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Department of Employment (Punjab)</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Punjab, India</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://www.pgrkam.com/</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Punjab, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Rajasthan Employment Department</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SRC-0346</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Rajasthan District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Department of Employment (Rajasthan)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Rajasthan, India</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://rajemployment.rajasthan.gov.in/</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Rajasthan, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.221897+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Kerala Employment Directorate</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SRC-0347</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Kerala District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Department of Employment (Kerala)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Kerala, India</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://www.employment.kerala.gov.in/</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Kerala, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.222464+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Tamil Nadu Employment (Velaivaaippu)</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SRC-0348</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Tamil Nadu District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Department of Employment (Tamil Nadu)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Tamil Nadu, India</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://tnvelaivaaippu.gov.in/</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Tamil Nadu, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.222464+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>UP Sewayojan Portal</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SRC-0349</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh District Employment Mission: Technical, Semi-Skilled &amp; Apprentice Drive</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Department of Employment (Uttar Pradesh)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>₹15,000 - ₹35,000 per month (State Minimum Wage / Apprenticeship)</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://sewayojan.up.nic.in/</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Employment Exchange, Rozgar Mela, Uttar Pradesh, Apprentice / Vocational</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-10-16T15:24:36.222464+00:00</t>
         </is>
       </c>
     </row>
@@ -5140,7 +7620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5362,7 +7842,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -5423,6 +7903,86 @@
       </c>
       <c r="D14" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SRC-STATE-PSC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>State Public Service Commissions (20 State PSCs)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SRC-STATE-SSSC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>State Subordinate Selection Boards (10 Boards)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SRC-BANK-REGULATORY</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Banking &amp; Financial Regulatory Institutions (8 Bodies)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SRC-STATE-EMPLOYMENT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>State Employment Exchanges &amp; Rozgar Portals (13 States)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete Archetype D Community and Social Listeners Engine with 7 channels and 4-tier pipeline
</commit_message>
<xml_diff>
--- a/module_1_scraping_engine/data/output/archetype_c_test_scraped_data.xlsx
+++ b/module_1_scraping_engine/data/output/archetype_c_test_scraped_data.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.237202+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.238203+00:00</t>
+          <t>2026-10-16T15:38:16.344491+00:00</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.643390+00:00</t>
+          <t>2026-10-16T15:38:16.883474+00:00</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:21.643390+00:00</t>
+          <t>2026-10-16T15:38:16.883474+00:00</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:22.416699+00:00</t>
+          <t>2026-10-16T15:38:17.666561+00:00</t>
         </is>
       </c>
     </row>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Latest Government Jobs October 2026 Notifications | 59915+ All India Vacancies</t>
+          <t>Latest Railway Jobs 2026 (7405+ Railway RRB Vacancies Open Now)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Government (Central / State Govt)</t>
+          <t>Government (RRB)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1891,17 +1891,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2015/10/Government-Jobs.html</t>
+          <t>https://www.indgovtjobs.in/2026/09/railway-jobs.html</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Government Job, Central / State Govt, Recruitment Notification</t>
+          <t>Government Job, RRB, Recruitment Notification</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -1918,12 +1918,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Govt Jobs for 10th 12th Pass</t>
+          <t>Govt Bank Jobs 2026: Apply Online, 3997+ Latest Vacancies</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Government (Central / State Govt)</t>
+          <t>Government (BANK)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1953,17 +1953,17 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2013/09/10th-12th-pass-govt-jobs.html</t>
+          <t>https://www.indgovtjobs.in/2026/08/bank-jobs.html</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Government Job, Central / State Govt, Recruitment Notification</t>
+          <t>Government Job, BANK, Recruitment Notification</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Govt Jobs for Graduates</t>
+          <t>Latest Government Jobs October 2026 Notifications | 59915+ All India Vacancies</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2013/09/government-jobs-for-graduates-2013-2014.html</t>
+          <t>https://www.indgovtjobs.in/2015/10/Government-Jobs.html</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Govt Jobs for Engineers</t>
+          <t>Govt Jobs for 10th 12th Pass</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2013/09/government-jobs-for-engineers-2013-2014.html</t>
+          <t>https://www.indgovtjobs.in/2013/09/10th-12th-pass-govt-jobs.html</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Govt Jobs for Diploma</t>
+          <t>Govt Jobs for Graduates</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2013/09/government-jobs-for-diploma-holders.html</t>
+          <t>https://www.indgovtjobs.in/2013/09/government-jobs-for-graduates-2013-2014.html</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Govt Jobs for ITI</t>
+          <t>Govt Jobs for Engineers</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2013/09/iti-fresher-jobs-2013-list.html</t>
+          <t>https://www.indgovtjobs.in/2013/09/government-jobs-for-engineers-2013-2014.html</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Govt Jobs for MBA</t>
+          <t>Govt Jobs for Diploma</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2014/08/MBA-Govt-Jobs.html</t>
+          <t>https://www.indgovtjobs.in/2013/09/government-jobs-for-diploma-holders.html</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Govt Jobs for MCA</t>
+          <t>Govt Jobs for ITI</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2014/08/MCA-Jobs.html</t>
+          <t>https://www.indgovtjobs.in/2013/09/iti-fresher-jobs-2013-list.html</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Govt Jobs for Law</t>
+          <t>Govt Jobs for MBA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/2015/07/Law-LLB-Govt-Jobs.html</t>
+          <t>https://www.indgovtjobs.in/2014/08/MBA-Govt-Jobs.html</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Railway Jobs</t>
+          <t>Govt Jobs for MCA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Government (RAILWAY)</t>
+          <t>Government (Central / State Govt)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2449,17 +2449,17 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.indgovtjobs.in/p/railway-jobs.html</t>
+          <t>https://www.indgovtjobs.in/2014/08/MCA-Jobs.html</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Government Job, RAILWAY, Recruitment Notification</t>
+          <t>Government Job, Central / State Govt, Recruitment Notification</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:23.555880+00:00</t>
+          <t>2026-10-16T15:38:18.728225+00:00</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:24.883630+00:00</t>
+          <t>2026-10-16T15:38:20.259352+00:00</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:24.884630+00:00</t>
+          <t>2026-10-16T15:38:20.260352+00:00</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:24.884630+00:00</t>
+          <t>2026-10-16T15:38:20.260352+00:00</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:24.884630+00:00</t>
+          <t>2026-10-16T15:38:20.260352+00:00</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:25.789582+00:00</t>
+          <t>2026-10-16T15:38:21.071502+00:00</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:25.789582+00:00</t>
+          <t>2026-10-16T15:38:21.071502+00:00</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:25.789582+00:00</t>
+          <t>2026-10-16T15:38:21.071502+00:00</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:25.789582+00:00</t>
+          <t>2026-10-16T15:38:21.071502+00:00</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:25.789582+00:00</t>
+          <t>2026-10-16T15:38:21.071502+00:00</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:30.349128+00:00</t>
+          <t>2026-10-16T15:38:25.473896+00:00</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:30.349128+00:00</t>
+          <t>2026-10-16T15:38:25.474565+00:00</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:30.349128+00:00</t>
+          <t>2026-10-16T15:38:25.474565+00:00</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:30.349958+00:00</t>
+          <t>2026-10-16T15:38:25.474565+00:00</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943051+00:00</t>
+          <t>2026-10-16T15:38:30.041918+00:00</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943051+00:00</t>
+          <t>2026-10-16T15:38:30.041918+00:00</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943051+00:00</t>
+          <t>2026-10-16T15:38:30.041918+00:00</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943051+00:00</t>
+          <t>2026-10-16T15:38:30.041918+00:00</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943051+00:00</t>
+          <t>2026-10-16T15:38:30.041918+00:00</t>
         </is>
       </c>
     </row>
@@ -3637,7 +3637,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.943608+00:00</t>
+          <t>2026-10-16T15:38:30.043218+00:00</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.043746+00:00</t>
         </is>
       </c>
     </row>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.044329+00:00</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:34.944113+00:00</t>
+          <t>2026-10-16T15:38:30.044329+00:00</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:35.470873+00:00</t>
+          <t>2026-10-16T15:38:30.537431+00:00</t>
         </is>
       </c>
     </row>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:35.470873+00:00</t>
+          <t>2026-10-16T15:38:30.537431+00:00</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:35.470873+00:00</t>
+          <t>2026-10-16T15:38:30.537431+00:00</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:35.470873+00:00</t>
+          <t>2026-10-16T15:38:30.537431+00:00</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.171805+00:00</t>
+          <t>2026-10-16T15:38:31.108371+00:00</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.171805+00:00</t>
+          <t>2026-10-16T15:38:31.108371+00:00</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.171805+00:00</t>
+          <t>2026-10-16T15:38:31.108371+00:00</t>
         </is>
       </c>
     </row>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5435,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5745,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215385+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5869,7 +5869,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.215972+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217136+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -5993,7 +5993,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217136+00:00</t>
+          <t>2026-10-16T15:38:31.109358+00:00</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6117,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6241,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6427,7 +6427,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6489,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.217821+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6737,7 +6737,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6799,7 +6799,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6861,7 +6861,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.219485+00:00</t>
+          <t>2026-10-16T15:38:31.110358+00:00</t>
         </is>
       </c>
     </row>
@@ -7047,7 +7047,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7357,7 +7357,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7419,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.221897+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.222464+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7543,7 +7543,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.222464+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>
@@ -7605,7 +7605,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:36.222464+00:00</t>
+          <t>2026-10-16T15:38:31.111357+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>